<commit_message>
feat(F-NAR-019): ATOM-EMO.LEX.002-06 Chouchou et la petite fleur
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-EMO.LEX.002-06.xlsx
+++ b/stories/arbres/ATOM-EMO.LEX.002-06.xlsx
@@ -671,7 +671,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>jardin, puis salon</t>
+          <t>jardin, puis salon, haie, fleur, terre, verre, tige, crayon, papier, table, vitre</t>
         </is>
       </c>
     </row>
@@ -683,7 +683,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Chouchou, maman, papa</t>
+          <t>Chouchou, papa, maman</t>
         </is>
       </c>
     </row>
@@ -841,7 +841,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Le vent couche la petite fleur de Chouchou. Il dit qu'il est triste. Il demande un câlin. Plus tard, son dessin se déchire. Il nomme encore la tristesse.</t>
+          <t>La terre du jardin sent le soleil. Près des fleurs, un éclat de haie luit. Chouchou veut donner l'eau, maintenant. Le vent couche la tige. Poitrine trop vite. Sourire parti. Yeux chauds. Papa s'accroupit. Je suis triste. Un câlin. Merci vécu. Deuxième ruse : le dessin se déchire au salon. Il refuse de foncer. Un éclat de haie tient près des fleurs.</t>
         </is>
       </c>
     </row>
@@ -1184,17 +1184,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Un escargot avance sur la pierre. Sa coquille est brune, toute petite. La terre est fraîche sous les doigts. Les feuilles bougent, tout doucement. Un bâton marque un trou dans la terre. Chouchou, ta fleur a de l'eau ? Oui. Un peu. Le vent arrive. On reste près du mur. D'accord, papa. En ce moment, Chouchou regarde sa fleur. La tige est verte, encore fine. Une petite tête jaune se tient droite. Elle est belle, maman. Elle est belle, oui. Le vent pousse les feuilles. La tige se couche dans la terre. Ma fleur... Parce que la fleur est couchée. Chouchou sent sa gorge serrée. Ses yeux deviennent chauds. Une larme tombe. Je suis triste. Tu es triste. C'est permis. Pleurer est permis. Chouchou pleure un peu. Les larmes coulent. Elles sont chaudes. Je t'écoute, Chouchou. Je veux un câlin. Viens. Un câlin. Maman ouvre les bras. Chouchou se blottit. Le câlin est chaud. Le gilet de maman sent l'herbe. Tu as dit : je suis triste. Bravo. Tu as demandé un câlin. Pleurer est permis, Chouchou. Le câlin aide. Oui. Le câlin aide. Plus tard, au salon. Une feuille de papier est sur la table. Le crayon rouge a roulé près du bord. Le dessin de Chouchou se déchire un peu. Un coin se fend, tout doucement. Chouchou sent encore sa gorge. Je suis triste. Tu es triste. C'est permis. Pleurer est permis. Je veux un câlin. Viens. Un câlin. Papa le serre. Ses épaules se desserrent. Bravo. Tu as dit tes larmes. On peut demander un câlin. La fleur, puis le dessin. La fleur, c'était pareil. L'escargot n'est plus sur la pierre.</t>
+          <t>La terre du jardin sent le soleil. Ça sent la terre, papa. Tu la sens, la terre chaude ? Oui, papa. Chouchou connaît ce jardin, ses coins, ses odeurs. Cette fin de matin, un coin brille autrement. Un vélo passe, très loin, derrière la haie. Tu entends le vélo, Chouchou ? Oui, maman. Près des fleurs, un éclat de haie luit. Il brille, maman. Tu le vois, le petit point ? Oui, sur la haie. La petite fleur attend dans la terre. La tige est verte, un peu fine. Une tête jaune se tient droite. Elle est belle, Chouchou ? Elle est belle, oui. Chouchou tient un verre d'eau, un peu lourd. C'est pour ma fleur. Tu lui donnes l'eau, Chouchou ? Oui, maintenant ! En ce moment, Chouchou penche le verre. Une goutte tombe près de la tige. Bois, petite fleur. Le vent arrive, Chouchou. On reste près de la haie ? Oui, on reste. Le vent pousse les branches de la haie. La tige se couche dans la terre. Ma fleur ! La tête jaune touche la terre humide. Elle est par terre ! Chouchou veut la redresser, tout de suite. Je la remets, maintenant ! Il tire trop vite sur la tige. La tige plie, plus bas qu'avant. Oh. Le sourire de Chouchou disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Sa gorge se serre. Ses yeux deviennent chauds. Une larme tombe sur le verre. Ses épaules tombent un peu. Papa s'accroupit à la même hauteur. Tu vois la fleur, Chouchou ? Oui, papa. Tes yeux sont chauds, Chouchou ? Un peu, maman. Je suis triste. Maman s'accroupit aussi, près de lui. Je veux un câlin. Viens. Maman ouvre les bras. Chouchou se blottit contre le gilet. Le gilet sent l'herbe chaude. On reste un peu ? Oui, papa. L'éclat de haie tremble, puis tient. La tige reste couchée, un peu. Elle est molle. On la verra tout à l'heure. On rentre un moment ? Oui.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Un escargot avance sur la pierre. Sa coquille est brune, toute petite. La terre est fraîche sous les doigts. Les feuilles bougent, tout doucement. Un bâton marque un trou dans la terre. Chouchou, ta fleur a de l'eau ? Oui. Un peu. Le vent arrive. On reste près du mur. D'accord, papa. En ce moment, Chouchou regarde sa fleur. La tige est verte, encore fine. Une petite tête jaune se tient droite. Elle est belle, maman. Elle est belle, oui. Le vent pousse les feuilles. La tige se couche dans la terre. Ma fleur... Parce que la fleur est couchée. Chouchou sent sa gorge serrée. Ses yeux deviennent chauds. Une larme tombe. Je suis triste. Tu es triste. C'est permis. Pleurer est permis. Chouchou pleure un peu. Les larmes coulent. Elles sont chaudes. Je t'écoute, Chouchou. Je veux un câlin. Viens. Un câlin. Maman ouvre les bras. Chouchou se blottit. Le câlin est chaud. Le gilet de maman sent l'herbe. Tu as dit : je suis triste. Bravo. Tu as demandé un câlin. Pleurer est permis, Chouchou. Le câlin aide. Oui. Le câlin aide. Plus tard, au salon. Une feuille de papier est sur la table. Le crayon rouge a roulé près du bord. Le dessin de Chouchou se déchire un peu. Un coin se fend, tout doucement. Chouchou sent encore sa gorge. Je suis triste. Tu es triste. C'est permis. Pleurer est permis. Je veux un câlin. Viens. Un câlin. Papa le serre. Ses épaules se desserrent. Bravo. Tu as dit tes larmes. On peut demander un câlin. La fleur, puis le dessin. La fleur, c'était pareil. L'escargot n'est plus sur la pierre.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;La terre du jardin sent le soleil. Ça sent la terre, papa. Tu la sens, la terre chaude ? Oui, papa. Chouchou connaît ce jardin, ses coins, ses odeurs. Cette fin de matin, un coin brille autrement. Un vélo passe, très loin, derrière la haie. Tu entends le vélo, Chouchou ? Oui, maman. Près des fleurs, un &lt;emphasis level="moderate"&gt;éclat de haie&lt;/emphasis&gt; luit. Il brille, maman. Tu le vois, le petit point ? Oui, sur la haie. La petite fleur attend dans la terre. La tige est verte, un peu fine. Une tête jaune se tient droite. Elle est belle, Chouchou ? Elle est belle, oui. Chouchou tient un verre d'eau, un peu lourd. C'est pour ma fleur. Tu lui donnes l'eau, Chouchou ? Oui, maintenant ! En ce moment, Chouchou penche le verre. Une goutte tombe près de la tige. Bois, petite fleur. Le vent arrive, Chouchou. On reste près de la haie ? Oui, on reste. Le vent pousse les branches de la haie. La tige se couche dans la terre. Ma fleur ! La tête jaune touche la terre humide. Elle est par terre ! Chouchou veut la redresser, tout de suite. Je la remets, maintenant ! Il tire trop vite sur la tige. La tige plie, plus bas qu'avant. Oh. Le sourire de Chouchou disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Sa gorge se serre. Ses yeux deviennent chauds. Une larme tombe sur le verre. Ses épaules tombent un peu. Papa s'accroupit à la même hauteur. Tu vois la fleur, Chouchou ? Oui, papa. Tes yeux sont chauds, Chouchou ? Un peu, maman. Je suis triste. Maman s'accroupit aussi, près de lui. Je veux un câlin. Viens. Maman ouvre les bras. Chouchou se blottit contre le gilet. Le gilet sent l'herbe chaude. On reste un peu ? Oui, papa. L'éclat de haie tremble, puis tient. La tige reste couchée, un peu. Elle est molle. On la verra tout à l'heure. On rentre un moment ? Oui.&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Félix a planté une petite fleur dans le jardin. Le vent a couché la tige. Félix sent sa gorge serrée. Ses yeux deviennent chauds. Une larme tombe. Félix dit : je suis &lt;emphasis&gt;triste&lt;/emphasis&gt;. Maman arrive près de lui. Maman dit : pleurer est permis. Félix pleure un peu. Les larmes coulent. Puis Félix dit : je veux un câlin. Maman ouvre les bras. Félix se blottit. Le câlin est chaud. Parce que la fleur est couchée, Félix est triste. Être triste, c'est permis. Plus tard, au salon, le dessin de Félix se déchire un peu. Félix sent encore sa gorge. Il dit : je suis triste. Papa dit : pleurer est permis. Félix demande un câlin. Papa le serre. Ses épaules se desserrent. Même leçon, autre moment. On nomme. On peut pleurer. On demande un câlin. [pause]</t>
+          <t>La terre du jardin sent le soleil. Ça sent la terre, papa. Tu la sens, la terre chaude ? Oui, papa. Chouchou connaît ce jardin, ses coins, ses odeurs. Cette fin de matin, un coin brille autrement. Un vélo passe, très loin, derrière la haie. Tu entends le vélo, Chouchou ? Oui, maman. Près des fleurs, un &lt;emphasis&gt;éclat de haie&lt;/emphasis&gt; luit. Il brille, maman. Tu le vois, le petit point ? Oui, sur la haie. La petite fleur attend dans la terre. La tige est verte, un peu fine. Une tête jaune se tient droite. Elle est belle, Chouchou ? Elle est belle, oui. Chouchou tient un verre d'eau, un peu lourd. C'est pour ma fleur. Tu lui donnes l'eau, Chouchou ? Oui, maintenant ! En ce moment, Chouchou penche le verre. Une goutte tombe près de la tige. Bois, petite fleur. Le vent arrive, Chouchou. On reste près de la haie ? Oui, on reste. Le vent pousse les branches de la haie. La tige se couche dans la terre. Ma fleur ! La tête jaune touche la terre humide. Elle est par terre ! Chouchou veut la redresser, tout de suite. Je la remets, maintenant ! Il tire trop vite sur la tige. La tige plie, plus bas qu'avant. Oh. Le sourire de Chouchou disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Sa gorge se serre. Ses yeux deviennent chauds. Une larme tombe sur le verre. Ses épaules tombent un peu. Papa s'accroupit à la même hauteur. Tu vois la fleur, Chouchou ? Oui, papa. Tes yeux sont chauds, Chouchou ? Un peu, maman. Je suis triste. Maman s'accroupit aussi, près de lui. Je veux un câlin. Viens. Maman ouvre les bras. Chouchou se blottit contre le gilet. Le gilet sent l'herbe chaude. On reste un peu ? Oui, papa. L'éclat de haie tremble, puis tient. La tige reste couchée, un peu. Elle est molle. On la verra tout à l'heure. On rentre un moment ? Oui. [pause]</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -1241,7 +1241,7 @@
         </is>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>148</v>
+        <v>142</v>
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
@@ -1249,7 +1249,7 @@
         </is>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>0.96</v>
+        <v>0.98</v>
       </c>
       <c r="AB2" s="2" t="n">
         <v>1.12</v>
@@ -1275,30 +1275,30 @@
       </c>
       <c r="AH2" s="2" t="inlineStr">
         <is>
-          <t>triste</t>
+          <t>éclat de haie</t>
         </is>
       </c>
       <c r="AI2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="AJ2" s="2" t="n">
-        <v>400</v>
+        <v>500</v>
       </c>
       <c r="AK2" s="2" t="n">
-        <v>280</v>
+        <v>260</v>
       </c>
       <c r="AL2" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>warm</t>
         </is>
       </c>
       <c r="AM2" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>storytelling</t>
         </is>
       </c>
       <c r="AN2" s="2" t="n">
-        <v>0.333</v>
+        <v>0.36</v>
       </c>
       <c r="AO2" s="2" t="inlineStr"/>
       <c r="AP2" s="2" t="inlineStr">
@@ -1307,10 +1307,10 @@
         </is>
       </c>
       <c r="AQ2" s="2" t="n">
-        <v>0.96</v>
+        <v>0.98</v>
       </c>
       <c r="AR2" s="2" t="n">
-        <v>0.96</v>
+        <v>0.98</v>
       </c>
       <c r="AS2" s="2" t="n">
         <v>100</v>
@@ -1321,65 +1321,77 @@
       <c r="AU2" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV2" s="2" t="inlineStr"/>
+      <c r="AV2" s="2" t="inlineStr">
+        <is>
+          <t>arc=installation; intention=émerveiller puis tendre; emotion=impatience puis tristesse; intensite=2; destinataire=enfant; sous_texte=il_veut_donner_l_eau_maintenant; tempo=naturel puis resserré; sourire=léger puis aucun; respiration=ample puis retenue</t>
+        </is>
+      </c>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|Un escargot avance sur la pierre.
-narrateur|Sa coquille est brune, toute petite.
-narrateur|La terre est fraîche sous les doigts.
-narrateur|Les feuilles bougent, tout doucement.
-narrateur|Un bâton marque un trou dans la terre.
-maman|Chouchou, ta fleur a de l'eau ?
-enfant-m|Oui. Un peu.
-papa|Le vent arrive. On reste près du mur.
-enfant-m|D'accord, papa.
-narrateur|En ce moment, Chouchou regarde sa fleur.
-narrateur|La tige est verte, encore fine.
-narrateur|Une petite tête jaune se tient droite.
-enfant-m|Elle est belle, maman.
-maman|Elle est belle, oui.
-narrateur|Le vent pousse les feuilles.
+          <t>narrateur|La terre du jardin sent le soleil.
+enfant-m|Ça sent la terre, papa.
+papa|Tu la sens, la terre chaude ?
+enfant-m|Oui, papa.
+narrateur|Chouchou connaît ce jardin, ses coins, ses odeurs.
+narrateur|Cette fin de matin, un coin brille autrement.
+narrateur|Un vélo passe, très loin, derrière la haie.
+maman|Tu entends le vélo, Chouchou ?
+enfant-m|Oui, maman.
+narrateur|Près des fleurs, un éclat de haie luit.
+enfant-m|Il brille, maman.
+maman|Tu le vois, le petit point ?
+enfant-m|Oui, sur la haie.
+narrateur|La petite fleur attend dans la terre.
+narrateur|La tige est verte, un peu fine.
+enfant-m|Une tête jaune se tient droite.
+papa|Elle est belle, Chouchou ?
+enfant-m|Elle est belle, oui.
+narrateur|Chouchou tient un verre d'eau, un peu lourd.
+enfant-m|C'est pour ma fleur.
+maman|Tu lui donnes l'eau, Chouchou ?
+enfant-m|Oui, maintenant !
+narrateur|En ce moment, Chouchou penche le verre.
+narrateur|Une goutte tombe près de la tige.
+enfant-m|Bois, petite fleur.
+papa|Le vent arrive, Chouchou.
+enfant-m|On reste près de la haie ?
+papa|Oui, on reste.
+narrateur|Le vent pousse les branches de la haie.
 narrateur|La tige se couche dans la terre.
-enfant-m|Ma fleur...
-narrateur|Parce que la fleur est couchée.
-narrateur|Chouchou sent sa gorge serrée.
+enfant-m|Ma fleur !
+narrateur|La tête jaune touche la terre humide.
+enfant-m|Elle est par terre !
+narrateur|Chouchou veut la redresser, tout de suite.
+enfant-m|Je la remets, maintenant !
+narrateur|Il tire trop vite sur la tige.
+narrateur|La tige plie, plus bas qu'avant.
+enfant-m|Oh.
+narrateur|Le sourire de Chouchou disparaît.
+narrateur|Dans sa poitrine, l'envie et l'inquiétude se bousculent.
+narrateur|Sa gorge se serre.
 narrateur|Ses yeux deviennent chauds.
-narrateur|Une larme tombe.
+narrateur|Une larme tombe sur le verre.
+narrateur|Ses épaules tombent un peu.
+narrateur|Papa s'accroupit à la même hauteur.
+papa|Tu vois la fleur, Chouchou ?
+enfant-m|Oui, papa.
+maman|Tes yeux sont chauds, Chouchou ?
+enfant-m|Un peu, maman.
 enfant-m|Je suis triste.
-maman|Tu es triste. C'est permis.
-maman|Pleurer est permis.
-narrateur|Chouchou pleure un peu.
-narrateur|Les larmes coulent. Elles sont chaudes.
-papa|Je t'écoute, Chouchou.
+narrateur|Maman s'accroupit aussi, près de lui.
 enfant-m|Je veux un câlin.
-maman|Viens. Un câlin.
+maman|Viens.
 narrateur|Maman ouvre les bras.
-narrateur|Chouchou se blottit.
-narrateur|Le câlin est chaud.
-narrateur|Le gilet de maman sent l'herbe.
-maman|Tu as dit : je suis triste.
-maman|Bravo. Tu as demandé un câlin.
-papa|Pleurer est permis, Chouchou.
-enfant-m|Le câlin aide.
-maman|Oui. Le câlin aide.
-narrateur|Plus tard, au salon.
-narrateur|Une feuille de papier est sur la table.
-narrateur|Le crayon rouge a roulé près du bord.
-narrateur|Le dessin de Chouchou se déchire un peu.
-narrateur|Un coin se fend, tout doucement.
-narrateur|Chouchou sent encore sa gorge.
-enfant-m|Je suis triste.
-papa|Tu es triste. C'est permis.
-papa|Pleurer est permis.
-enfant-m|Je veux un câlin.
-papa|Viens. Un câlin.
-narrateur|Papa le serre.
-narrateur|Ses épaules se desserrent.
-maman|Bravo. Tu as dit tes larmes.
-maman|On peut demander un câlin.
-enfant-m|La fleur, puis le dessin.
-papa|La fleur, c'était pareil.
-narrateur|L'escargot n'est plus sur la pierre.</t>
+narrateur|Chouchou se blottit contre le gilet.
+narrateur|Le gilet sent l'herbe chaude.
+papa|On reste un peu ?
+enfant-m|Oui, papa.
+narrateur|L'éclat de haie tremble, puis tient.
+narrateur|La tige reste couchée, un peu.
+enfant-m|Elle est molle.
+papa|On la verra tout à l'heure.
+maman|On rentre un moment ?
+enfant-m|Oui.</t>
         </is>
       </c>
       <c r="AX2" t="inlineStr">
@@ -1416,12 +1428,12 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Chouchou a les yeux chauds. Que dit-il ?</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;&lt;emphasis level="moderate"&gt;Chouchou&lt;/emphasis&gt; a les yeux chauds. Que dit-il ?&lt;/prosody&gt;&lt;break time="700ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>Félix a les yeux chauds. Que dit-il ?</t>
+          <t>&lt;soft&gt;&lt;slow&gt;&lt;emphasis&gt;Chouchou&lt;/emphasis&gt; a les yeux chauds. Que dit-il ?&lt;/slow&gt;&lt;/soft&gt; [pause]</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -1446,7 +1458,7 @@
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>Félix peut demander un câlin. Que dit-il ?</t>
+          <t>Chouchou peut demander un câlin. Que dit-il ?</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr"/>
@@ -1484,18 +1496,18 @@
         </is>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>130</v>
+        <v>120</v>
       </c>
       <c r="Z3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>slow</t>
         </is>
       </c>
       <c r="AA3" s="2" t="n">
-        <v>0.9</v>
+        <v>0.86</v>
       </c>
       <c r="AB3" s="2" t="n">
-        <v>1.24</v>
+        <v>1.27</v>
       </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
@@ -1510,34 +1522,38 @@
       <c r="AE3" s="2" t="inlineStr"/>
       <c r="AF3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>soft</t>
         </is>
       </c>
       <c r="AG3" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH3" s="2" t="inlineStr"/>
+        <v>-2</v>
+      </c>
+      <c r="AH3" s="2" t="inlineStr">
+        <is>
+          <t>Chouchou</t>
+        </is>
+      </c>
       <c r="AI3" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ3" s="2" t="n">
-        <v>250</v>
+        <v>700</v>
       </c>
       <c r="AK3" s="2" t="n">
-        <v>280</v>
+        <v>320</v>
       </c>
       <c r="AL3" s="2" t="inlineStr">
         <is>
-          <t>warm</t>
+          <t>focused</t>
         </is>
       </c>
       <c r="AM3" s="2" t="inlineStr">
         <is>
-          <t>rise</t>
+          <t>rising</t>
         </is>
       </c>
       <c r="AN3" s="2" t="n">
-        <v>0.333</v>
+        <v>0.32</v>
       </c>
       <c r="AO3" s="2" t="inlineStr"/>
       <c r="AP3" s="2" t="inlineStr">
@@ -1546,28 +1562,29 @@
         </is>
       </c>
       <c r="AQ3" s="2" t="n">
-        <v>0.9</v>
+        <v>0.86</v>
       </c>
       <c r="AR3" s="2" t="n">
-        <v>0.9</v>
+        <v>0.86</v>
       </c>
       <c r="AS3" s="2" t="n">
-        <v>100</v>
+        <v>82</v>
       </c>
       <c r="AT3" s="2" t="n">
         <v>50</v>
       </c>
       <c r="AU3" s="2" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="AV3" s="2" t="inlineStr">
         <is>
-          <t>question d'écoute, ne change pas le cours</t>
+          <t>arc=indice; intention=faire_deviner; emotion=attention; intensite=1; destinataire=enfant; sous_texte=chouchou_a_les_yeux_chauds_que_dit_il; tempo=suspendu; sourire=aucun; respiration=courte_avant_question</t>
         </is>
       </c>
       <c r="AW3" t="inlineStr">
         <is>
-          <t>narrateur|Chouchou a les yeux chauds. Que dit-il ?</t>
+          <t>narrateur|Chouchou a les yeux chauds.
+narrateur|Que dit-il ?</t>
         </is>
       </c>
     </row>
@@ -1594,17 +1611,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Chouchou sèche une larme avec sa manche. Je suis triste. Oui. Et pleurer est permis. Un câlin de papa ou maman aide. Bravo. Tu as dit ce que tu sentais. Tu veux encore un câlin ? Encore un peu. Papa le serre, sans se presser. La table est lisse sous la main.</t>
+          <t>Chouchou sèche une larme avec sa manche. Le câlin est chaud. Tes épaules se desserrent ? Un peu, maman. Ils restent accroupis près de la haie. On va au salon, Chouchou ? Oui. Chouchou veut courir vers la porte. Les mots se bousculent dans sa bouche. Le dessin, maintenant ! Il avance trop vite vers le seuil. Puis il s'arrête. Chouchou refuse de foncer. Il referme la bouche. Personne ne parle. Il observe la fleur, un instant. Il écoute le jardin. Tu restes un peu, Chouchou ? Oui, papa. Merci, Chouchou. Papa reste à la même hauteur. Le verre est tiède, sous les doigts. Il est vide. On marche sans se presser ? Oui, papa. Le ventre de Chouchou se desserre. Les épaules se relèvent un peu. On prend le crayon rouge ? Oui, pour la fleur. Ils passent la porte du salon. La table est là. Tu as de la place, Chouchou ? Oui, papa. Le crayon rouge attend près du bord. Tu fais ta fleur, Chouchou ? Oui, maman.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Chouchou sèche une larme avec sa manche. Je suis triste. Oui. Et pleurer est permis. Un câlin de papa ou maman aide. Bravo. Tu as dit ce que tu sentais. Tu veux encore un câlin ? Encore un peu. Papa le serre, sans se presser. La table est lisse sous la main.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Chouchou sèche une larme avec sa manche. Le &lt;emphasis level="moderate"&gt;câlin&lt;/emphasis&gt; est chaud. Tes épaules se desserrent ? Un peu, maman. Ils restent accroupis près de la haie. On va au salon, Chouchou ? Oui. Chouchou veut courir vers la porte. Les mots se bousculent dans sa bouche. Le dessin, maintenant ! Il avance trop vite vers le seuil. Puis il s'arrête. Chouchou refuse de foncer. Il referme la bouche. Personne ne parle. Il observe la fleur, un instant. Il écoute le jardin. Tu restes un peu, Chouchou ? Oui, papa. Merci, Chouchou. Papa reste à la même hauteur. Le verre est tiède, sous les doigts. Il est vide. On marche sans se presser ? Oui, papa. Le ventre de Chouchou se desserre. Les épaules se relèvent un peu. On prend le crayon rouge ? Oui, pour la fleur. Ils passent la porte du salon. La table est là. Tu as de la place, Chouchou ? Oui, papa. Le crayon rouge attend près du bord. Tu fais ta fleur, Chouchou ? Oui, maman.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Félix a nommé : &lt;emphasis&gt;triste&lt;/emphasis&gt;. Pleurer est permis. Un câlin de papa ou maman aide. [pause]</t>
+          <t>Chouchou sèche une larme avec sa manche. Le &lt;emphasis&gt;câlin&lt;/emphasis&gt; est chaud. Tes épaules se desserrent ? Un peu, maman. Ils restent accroupis près de la haie. On va au salon, Chouchou ? Oui. Chouchou veut courir vers la porte. Les mots se bousculent dans sa bouche. Le dessin, maintenant ! Il avance trop vite vers le seuil. Puis il s'arrête. Chouchou refuse de foncer. Il referme la bouche. Personne ne parle. Il observe la fleur, un instant. Il écoute le jardin. Tu restes un peu, Chouchou ? Oui, papa. Merci, Chouchou. Papa reste à la même hauteur. Le verre est tiède, sous les doigts. Il est vide. On marche sans se presser ? Oui, papa. Le ventre de Chouchou se desserre. Les épaules se relèvent un peu. On prend le crayon rouge ? Oui, pour la fleur. Ils passent la porte du salon. La table est là. Tu as de la place, Chouchou ? Oui, papa. Le crayon rouge attend près du bord. Tu fais ta fleur, Chouchou ? Oui, maman. [pause]</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -1651,7 +1668,7 @@
         </is>
       </c>
       <c r="Y4" s="2" t="n">
-        <v>148</v>
+        <v>140</v>
       </c>
       <c r="Z4" s="2" t="inlineStr">
         <is>
@@ -1659,10 +1676,10 @@
         </is>
       </c>
       <c r="AA4" s="2" t="n">
-        <v>0.96</v>
+        <v>0.97</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>1.12</v>
+        <v>1.14</v>
       </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
@@ -1685,30 +1702,30 @@
       </c>
       <c r="AH4" s="2" t="inlineStr">
         <is>
-          <t>triste</t>
+          <t>câlin</t>
         </is>
       </c>
       <c r="AI4" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ4" s="2" t="n">
-        <v>450</v>
+        <v>560</v>
       </c>
       <c r="AK4" s="2" t="n">
-        <v>280</v>
+        <v>270</v>
       </c>
       <c r="AL4" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>bright</t>
         </is>
       </c>
       <c r="AM4" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN4" s="2" t="n">
-        <v>0.333</v>
+        <v>0.35</v>
       </c>
       <c r="AO4" s="2" t="inlineStr"/>
       <c r="AP4" s="2" t="inlineStr">
@@ -1717,10 +1734,10 @@
         </is>
       </c>
       <c r="AQ4" s="2" t="n">
-        <v>0.96</v>
+        <v>0.97</v>
       </c>
       <c r="AR4" s="2" t="n">
-        <v>0.96</v>
+        <v>0.97</v>
       </c>
       <c r="AS4" s="2" t="n">
         <v>100</v>
@@ -1733,20 +1750,47 @@
       </c>
       <c r="AV4" s="2" t="inlineStr">
         <is>
-          <t>confirmation ; le moteur peut dire engine_ok/near avant ce chunk</t>
+          <t>arc=résolution; intention=faire_vivre_le_geste; emotion=retenue puis fierté_calme; intensite=2; destinataire=enfant; sous_texte=il_nomme_triste_il_demande_un_calin; tempo=naturel; sourire=léger; respiration=relâchée</t>
         </is>
       </c>
       <c r="AW4" t="inlineStr">
         <is>
           <t>narrateur|Chouchou sèche une larme avec sa manche.
-enfant-m|Je suis triste.
-maman|Oui. Et pleurer est permis.
-papa|Un câlin de papa ou maman aide.
-maman|Bravo. Tu as dit ce que tu sentais.
-maman|Tu veux encore un câlin ?
-enfant-m|Encore un peu.
-narrateur|Papa le serre, sans se presser.
-narrateur|La table est lisse sous la main.</t>
+enfant-m|Le câlin est chaud.
+maman|Tes épaules se desserrent ?
+enfant-m|Un peu, maman.
+narrateur|Ils restent accroupis près de la haie.
+papa|On va au salon, Chouchou ?
+enfant-m|Oui.
+narrateur|Chouchou veut courir vers la porte.
+narrateur|Les mots se bousculent dans sa bouche.
+enfant-m|Le dessin, maintenant !
+narrateur|Il avance trop vite vers le seuil.
+narrateur|Puis il s'arrête.
+narrateur|Chouchou refuse de foncer.
+narrateur|Il referme la bouche.
+narrateur|Personne ne parle.
+narrateur|Il observe la fleur, un instant.
+narrateur|Il écoute le jardin.
+papa|Tu restes un peu, Chouchou ?
+enfant-m|Oui, papa.
+papa|Merci, Chouchou.
+narrateur|Papa reste à la même hauteur.
+maman|Le verre est tiède, sous les doigts.
+enfant-m|Il est vide.
+papa|On marche sans se presser ?
+enfant-m|Oui, papa.
+narrateur|Le ventre de Chouchou se desserre.
+narrateur|Les épaules se relèvent un peu.
+maman|On prend le crayon rouge ?
+enfant-m|Oui, pour la fleur.
+narrateur|Ils passent la porte du salon.
+enfant-m|La table est là.
+papa|Tu as de la place, Chouchou ?
+enfant-m|Oui, papa.
+narrateur|Le crayon rouge attend près du bord.
+maman|Tu fais ta fleur, Chouchou ?
+enfant-m|Oui, maman.</t>
         </is>
       </c>
     </row>
@@ -1773,17 +1817,17 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Maman redresse la petite fleur. Un peu de terre autour de la tige. Elle se tient. Elle se tient, oui. Chouchou pose son dessin près de lui. Tu as bien demandé le câlin. Je suis moins triste. Le câlin est encore là. Ils restent près de la fleur, tout calmes.</t>
+          <t>Un papier blanc attend sur la table. Je dessine ma fleur. Le crayon rouge a un bout usé. Tu fais la tige, Chouchou ? Oui, papa. Chouchou trace une tige, trop vite. Et la tête jaune ! Il appuie trop fort sur le papier. Un coin du dessin se fend. Il se déchire ! Le papier s'ouvre un peu, net. Ma fleur ! Chouchou veut coller le coin, tout de suite. Je le tiens, maintenant ! Il avance les mains, trop vite. Puis il s'arrête net. Chouchou refuse de foncer, cette fois. Ses mains se ferment, puis s'ouvrent. Personne ne dit la suite. Il observe le dessin, un instant. Il écoute le salon, près de la table. Derrière la vitre, un éclat de haie luit. Là, sur la haie. Chouchou pose les mains à plat. Je veux un câlin. Viens. Papa le serre, sans se presser. Le coin est fendu. On le lisse un peu ? Oui, maman. Chouchou lisse le papier, sans se presser. On tient le coin ? Oui, papa. Le dessin reste, un peu fendu. Poumf. La tête jaune est là, Chouchou ? Oui, maman. Tu vois le point, Chouchou ? Oui, papa. Le crayon rouge a roulé près du bord.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Maman redresse la petite fleur. Un peu de terre autour de la tige. Elle se tient. Elle se tient, oui. Chouchou pose son dessin près de lui. Tu as bien demandé le câlin. Je suis moins triste. Le câlin est encore là. Ils restent près de la fleur, tout calmes.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Un papier blanc attend sur la table. Je dessine ma fleur. Le crayon rouge a un bout usé. Tu fais la tige, Chouchou ? Oui, papa. Chouchou trace une tige, trop vite. Et la tête jaune ! Il appuie trop fort sur le papier. Un coin du dessin se fend. Il se déchire ! Le papier s'ouvre un peu, net. Ma fleur ! Chouchou veut coller le coin, tout de suite. Je le tiens, maintenant ! Il avance les mains, trop vite. Puis il s'arrête net. Chouchou refuse de foncer, cette fois. Ses mains se ferment, puis s'ouvrent. Personne ne dit la suite. Il observe le dessin, un instant. Il écoute le salon, près de la table. Derrière la vitre, un &lt;emphasis level="moderate"&gt;éclat de haie&lt;/emphasis&gt; luit. Là, sur la haie. Chouchou pose les mains à plat. Je veux un câlin. Viens. Papa le serre, sans se presser. Le coin est fendu. On le lisse un peu ? Oui, maman. Chouchou lisse le papier, sans se presser. On tient le coin ? Oui, papa. Le dessin reste, un peu fendu. Poumf. La tête jaune est là, Chouchou ? Oui, maman. Tu vois le point, Chouchou ? Oui, papa. Le crayon rouge a roulé près du bord.&lt;/prosody&gt;&lt;break time="420ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Maman redresse la petite fleur. Félix pose son dessin près de lui. [pause]</t>
+          <t>Un papier blanc attend sur la table. Je dessine ma fleur. Le crayon rouge a un bout usé. Tu fais la tige, Chouchou ? Oui, papa. Chouchou trace une tige, trop vite. Et la tête jaune ! Il appuie trop fort sur le papier. Un coin du dessin se fend. Il se déchire ! Le papier s'ouvre un peu, net. Ma fleur ! Chouchou veut coller le coin, tout de suite. Je le tiens, maintenant ! Il avance les mains, trop vite. Puis il s'arrête net. Chouchou refuse de foncer, cette fois. Ses mains se ferment, puis s'ouvrent. Personne ne dit la suite. Il observe le dessin, un instant. Il écoute le salon, près de la table. Derrière la vitre, un &lt;emphasis&gt;éclat de haie&lt;/emphasis&gt; luit. Là, sur la haie. Chouchou pose les mains à plat. Je veux un câlin. Viens. Papa le serre, sans se presser. Le coin est fendu. On le lisse un peu ? Oui, maman. Chouchou lisse le papier, sans se presser. On tient le coin ? Oui, papa. Le dessin reste, un peu fendu. Poumf. La tête jaune est là, Chouchou ? Oui, maman. Tu vois le point, Chouchou ? Oui, papa. Le crayon rouge a roulé près du bord. [pause]</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -1830,7 +1874,7 @@
         </is>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
@@ -1838,10 +1882,10 @@
         </is>
       </c>
       <c r="AA5" s="2" t="n">
-        <v>0.96</v>
+        <v>1</v>
       </c>
       <c r="AB5" s="2" t="n">
-        <v>1.12</v>
+        <v>1.1</v>
       </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
@@ -1862,28 +1906,32 @@
       <c r="AG5" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AH5" s="2" t="inlineStr"/>
+      <c r="AH5" s="2" t="inlineStr">
+        <is>
+          <t>éclat de haie</t>
+        </is>
+      </c>
       <c r="AI5" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ5" s="2" t="n">
-        <v>450</v>
+        <v>420</v>
       </c>
       <c r="AK5" s="2" t="n">
-        <v>280</v>
+        <v>250</v>
       </c>
       <c r="AL5" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>lively</t>
         </is>
       </c>
       <c r="AM5" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>dynamic</t>
         </is>
       </c>
       <c r="AN5" s="2" t="n">
-        <v>0.333</v>
+        <v>0.37</v>
       </c>
       <c r="AO5" s="2" t="inlineStr"/>
       <c r="AP5" s="2" t="inlineStr">
@@ -1892,10 +1940,10 @@
         </is>
       </c>
       <c r="AQ5" s="2" t="n">
-        <v>0.96</v>
+        <v>1</v>
       </c>
       <c r="AR5" s="2" t="n">
-        <v>0.96</v>
+        <v>1</v>
       </c>
       <c r="AS5" s="2" t="n">
         <v>100</v>
@@ -1906,23 +1954,58 @@
       <c r="AU5" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV5" s="2" t="inlineStr"/>
+      <c r="AV5" s="2" t="inlineStr">
+        <is>
+          <t>arc=action; intention=entraîner; emotion=élan puis prudence; intensite=2; destinataire=enfant; sous_texte=le_dessin_se_dechire_il_refuse_de_foncer; tempo=vif puis posé; sourire=léger; respiration=courte</t>
+        </is>
+      </c>
       <c r="AW5" t="inlineStr">
         <is>
-          <t>narrateur|Maman redresse la petite fleur.
-narrateur|Un peu de terre autour de la tige.
-enfant-m|Elle se tient.
-maman|Elle se tient, oui.
-narrateur|Chouchou pose son dessin près de lui.
-papa|Tu as bien demandé le câlin.
-enfant-m|Je suis moins triste.
-maman|Le câlin est encore là.
-narrateur|Ils restent près de la fleur, tout calmes.</t>
+          <t>narrateur|Un papier blanc attend sur la table.
+enfant-m|Je dessine ma fleur.
+narrateur|Le crayon rouge a un bout usé.
+papa|Tu fais la tige, Chouchou ?
+enfant-m|Oui, papa.
+narrateur|Chouchou trace une tige, trop vite.
+enfant-m|Et la tête jaune !
+narrateur|Il appuie trop fort sur le papier.
+narrateur|Un coin du dessin se fend.
+enfant-m|Il se déchire !
+narrateur|Le papier s'ouvre un peu, net.
+enfant-m|Ma fleur !
+narrateur|Chouchou veut coller le coin, tout de suite.
+enfant-m|Je le tiens, maintenant !
+narrateur|Il avance les mains, trop vite.
+narrateur|Puis il s'arrête net.
+narrateur|Chouchou refuse de foncer, cette fois.
+narrateur|Ses mains se ferment, puis s'ouvrent.
+narrateur|Personne ne dit la suite.
+narrateur|Il observe le dessin, un instant.
+narrateur|Il écoute le salon, près de la table.
+narrateur|Derrière la vitre, un éclat de haie luit.
+enfant-m|Là, sur la haie.
+narrateur|Chouchou pose les mains à plat.
+enfant-m|Je veux un câlin.
+papa|Viens.
+narrateur|Papa le serre, sans se presser.
+enfant-m|Le coin est fendu.
+maman|On le lisse un peu ?
+enfant-m|Oui, maman.
+narrateur|Chouchou lisse le papier, sans se presser.
+papa|On tient le coin ?
+enfant-m|Oui, papa.
+narrateur|Le dessin reste, un peu fendu.
+enfant-m|Poumf.
+maman|La tête jaune est là, Chouchou ?
+enfant-m|Oui, maman.
+papa|Tu vois le point, Chouchou ?
+enfant-m|Oui, papa.
+narrateur|Le crayon rouge a roulé près du bord.</t>
         </is>
       </c>
       <c r="AX5" t="inlineStr">
         <is>
-          <t>jardin</t>
+          <t>papier</t>
         </is>
       </c>
     </row>
@@ -1949,17 +2032,17 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>J'ai dit : je suis triste. J'ai eu un câlin. Pleurer est permis. Bravo, Chouchou.</t>
+          <t>Ils reviennent près de la haie. Maman redresse un peu la tige. Elle se tient. Elle se tient, oui. Chouchou pose son dessin près de lui. Le coin est fendu, papa. Tu l'as vu, toi ? Oui, près de la tige. On est bien, ici. Chouchou tapote le papier du doigt. Il a une trace de crayon. Tu la vois, la trace ? Oui, maman. La fleur est restée, Chouchou. Oui, avec le dessin. Ça sent la terre, un peu tiède. Et l'herbe, maman. Oui, dans l'air. Le jardin est calme, Chouchou ? Oui, papa. La petite fleur reste dans la terre. Un éclat de haie tient près des fleurs.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>J'ai dit : je suis triste. J'ai eu un câlin. Pleurer est permis. Bravo, Chouchou.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Ils reviennent près de la haie. Maman redresse un peu la tige. Elle se tient. Elle se tient, oui. Chouchou pose son dessin près de lui. Le coin est fendu, papa. Tu l'as vu, toi ? Oui, près de la tige. On est bien, ici. Chouchou tapote le papier du doigt. Il a une trace de crayon. Tu la vois, la trace ? Oui, maman. La fleur est restée, Chouchou. Oui, avec le dessin. Ça sent la terre, un peu tiède. Et l'herbe, maman. Oui, dans l'air. Le jardin est calme, Chouchou ? Oui, papa. La petite fleur reste dans la terre. Un &lt;emphasis level="moderate"&gt;éclat de haie&lt;/emphasis&gt; tient près des fleurs.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;L'histoire est finie.&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Ils reviennent près de la haie. Maman redresse un peu la tige. Elle se tient. Elle se tient, oui. Chouchou pose son dessin près de lui. Le coin est fendu, papa. Tu l'as vu, toi ? Oui, près de la tige. On est bien, ici. Chouchou tapote le papier du doigt. Il a une trace de crayon. Tu la vois, la trace ? Oui, maman. La fleur est restée, Chouchou. Oui, avec le dessin. Ça sent la terre, un peu tiède. Et l'herbe, maman. Oui, dans l'air. Le jardin est calme, Chouchou ? Oui, papa. La petite fleur reste dans la terre. Un &lt;emphasis&gt;éclat de haie&lt;/emphasis&gt; tient près des fleurs.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -2006,18 +2089,18 @@
         </is>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>136</v>
+        <v>118</v>
       </c>
       <c r="Z6" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>slow</t>
         </is>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>0.92</v>
+        <v>0.85</v>
       </c>
       <c r="AB6" s="2" t="n">
-        <v>1.2</v>
+        <v>1.28</v>
       </c>
       <c r="AC6" s="2" t="inlineStr">
         <is>
@@ -2026,12 +2109,12 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>-2st</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
         <is>
-          <t>lower-pitch</t>
+          <t>low-pitch</t>
         </is>
       </c>
       <c r="AF6" s="2" t="inlineStr">
@@ -2040,17 +2123,21 @@
         </is>
       </c>
       <c r="AG6" s="2" t="n">
-        <v>-2</v>
-      </c>
-      <c r="AH6" s="2" t="inlineStr"/>
+        <v>-3</v>
+      </c>
+      <c r="AH6" s="2" t="inlineStr">
+        <is>
+          <t>éclat de haie</t>
+        </is>
+      </c>
       <c r="AI6" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ6" s="2" t="n">
-        <v>600</v>
+        <v>900</v>
       </c>
       <c r="AK6" s="2" t="n">
-        <v>280</v>
+        <v>340</v>
       </c>
       <c r="AL6" s="2" t="inlineStr">
         <is>
@@ -2059,11 +2146,11 @@
       </c>
       <c r="AM6" s="2" t="inlineStr">
         <is>
-          <t>fall</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN6" s="2" t="n">
-        <v>0.333</v>
+        <v>0.31</v>
       </c>
       <c r="AO6" s="2" t="inlineStr"/>
       <c r="AP6" s="2" t="inlineStr">
@@ -2072,27 +2159,54 @@
         </is>
       </c>
       <c r="AQ6" s="2" t="n">
-        <v>0.92</v>
+        <v>0.85</v>
       </c>
       <c r="AR6" s="2" t="n">
-        <v>0.92</v>
+        <v>0.85</v>
       </c>
       <c r="AS6" s="2" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="AT6" s="2" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="AU6" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="AV6" s="2" t="inlineStr"/>
+        <v>12</v>
+      </c>
+      <c r="AV6" s="2" t="inlineStr">
+        <is>
+          <t>arc=retour; intention=refermer; emotion=tendresse_et_fierté_calme; intensite=1; destinataire=enfant; sous_texte=l_eclat_du_debut_tient_pres_des_fleurs; tempo=posé; sourire=léger; respiration=ample</t>
+        </is>
+      </c>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>enfant-m|J'ai dit : je suis triste.
-enfant-m|J'ai eu un câlin.
-maman|Pleurer est permis.
-papa|Bravo, Chouchou.</t>
+          <t>narrateur|Ils reviennent près de la haie.
+narrateur|Maman redresse un peu la tige.
+enfant-m|Elle se tient.
+maman|Elle se tient, oui.
+narrateur|Chouchou pose son dessin près de lui.
+enfant-m|Le coin est fendu, papa.
+papa|Tu l'as vu, toi ?
+enfant-m|Oui, près de la tige.
+maman|On est bien, ici.
+narrateur|Chouchou tapote le papier du doigt.
+enfant-m|Il a une trace de crayon.
+maman|Tu la vois, la trace ?
+enfant-m|Oui, maman.
+papa|La fleur est restée, Chouchou.
+enfant-m|Oui, avec le dessin.
+narrateur|Ça sent la terre, un peu tiède.
+enfant-m|Et l'herbe, maman.
+maman|Oui, dans l'air.
+papa|Le jardin est calme, Chouchou ?
+enfant-m|Oui, papa.
+narrateur|La petite fleur reste dans la terre.
+narrateur|Un éclat de haie tient près des fleurs.</t>
+        </is>
+      </c>
+      <c r="AX6" t="inlineStr">
+        <is>
+          <t>jardin</t>
         </is>
       </c>
     </row>
@@ -2113,7 +2227,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A7"/>
+  <dimension ref="A1:A8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2163,6 +2277,13 @@
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>